<commit_message>
Update dataset and datasheet generation
</commit_message>
<xml_diff>
--- a/backend/user_logs.xlsx
+++ b/backend/user_logs.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="24">
   <si>
     <t>Timestamp</t>
   </si>
@@ -53,6 +53,9 @@
   </si>
   <si>
     <t>2026-05-06 21:29:01</t>
+  </si>
+  <si>
+    <t>2026-05-13 21:48:41</t>
   </si>
   <si>
     <t>LOGIN</t>
@@ -440,7 +443,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -465,13 +468,13 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -479,16 +482,16 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -496,13 +499,13 @@
         <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -510,13 +513,13 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -524,16 +527,16 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -541,13 +544,13 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -555,13 +558,13 @@
         <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -569,13 +572,24 @@
         <v>12</v>
       </c>
       <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" t="s">
         <v>13</v>
       </c>
-      <c r="C9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D9" t="s">
-        <v>21</v>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>